<commit_message>
Use supplied working ZIP as base for official college data update
</commit_message>
<xml_diff>
--- a/sample_data/it_presentation.xlsx
+++ b/sample_data/it_presentation.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dr. Anjali Deshmukh</t>
+          <t>Dr.Vidya Kubde</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -595,7 +595,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prof. Rahul Patil</t>
+          <t>Dr.R. V. Bhaskarwar</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prof. Aniket Joshi</t>
+          <t>Mrs. A. D. Mhatre</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -687,7 +687,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Prof. Sneha Joshi</t>
+          <t>Mrs. G.M.Arwindekar</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -733,7 +733,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Prof. Riya Kulkarni</t>
+          <t>Mr.J. R. Gaidhane</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -779,7 +779,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Prof. Amit Shah</t>
+          <t>Dr. R.A.Jolhe</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -825,7 +825,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Prof. Pooja Kulkarni</t>
+          <t>Ms. D. P. Kadam</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -871,7 +871,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Prof. Sahil Desai</t>
+          <t>Mr. S. U. Kumane</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -917,7 +917,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Prof. Vikram More</t>
+          <t>Mrs. K. P. Rane</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -963,7 +963,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prof. Sanika Rane</t>
+          <t>Mrs. H. A.Khot</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Prof. Omkar Kale</t>
+          <t>Mrs. A. R. Rahude</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dr. Meera Nair</t>
+          <t>Mrs. N.Y. Moharkar</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prof. Sandeep Jadhav</t>
+          <t>Mrs. J. S. Phonde</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Prof. Kunal Patil</t>
+          <t>Mr. Krushna Jadhav</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prof. Neha Desai</t>
+          <t>Mrs. Angel Bency</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Prof. Neelam Shah</t>
+          <t>Mrs. Karishma Shelar</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Prof. Kiran Rao</t>
+          <t>Mrs. Vaishali Korade</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dr. Priya Menon</t>
+          <t>Pallavi M.N.</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Prof. Varun Nair</t>
+          <t>Bipasha</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Prof. Aditya Gokhale</t>
+          <t>Priya Jadhav</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dr. Snehal Shinde</t>
+          <t>Pankaj Rathod</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Prof. Akash Pawar</t>
+          <t>Harshali Vihire</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dr. Shreya Kulkarni</t>
+          <t>Reshma</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Prof. Nikhil Sawant</t>
+          <t>Sample Professor 01</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Prof. Tanvi Rao</t>
+          <t>Sample Professor 02</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prof. Kavita Iyer</t>
+          <t>Sample Professor 03</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Prof. Pranav More</t>
+          <t>Sample Professor 04</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Prof. Rohit Bhosale</t>
+          <t>Sample Professor 05</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dr. Aditi Naik</t>
+          <t>Sample Professor 06</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Prof. Rohini Jadhav</t>
+          <t>Sample Professor 07</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Prof. Sameer Pawar</t>
+          <t>Sample Professor 08</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Prof. Rutuja More</t>
+          <t>Sample Professor 09</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dr. Harsh Mehta</t>
+          <t>Sample Professor 10</t>
         </is>
       </c>
       <c r="C34" t="n">

</xml_diff>